<commit_message>
feat: add demo files on main page and some changes
</commit_message>
<xml_diff>
--- a/data/Сажида (русс)/1. Личные местоимения.xlsx
+++ b/data/Сажида (русс)/1. Личные местоимения.xlsx
@@ -45,9 +45,6 @@
     <t>أَنْتِ</t>
   </si>
   <si>
-    <t>أَنْتُمَا</t>
-  </si>
-  <si>
     <t>أَنْتُنَّ</t>
   </si>
   <si>
@@ -58,6 +55,39 @@
   </si>
   <si>
     <t>نَحْنُ</t>
+  </si>
+  <si>
+    <t>Она</t>
+  </si>
+  <si>
+    <t>Мы</t>
+  </si>
+  <si>
+    <t>Я</t>
+  </si>
+  <si>
+    <t>Вы обе</t>
+  </si>
+  <si>
+    <t>Вы оба</t>
+  </si>
+  <si>
+    <t>أَنْتُمَا (жр)</t>
+  </si>
+  <si>
+    <r>
+      <t xml:space="preserve">أَنْتُمَا </t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="8"/>
+        <color theme="1"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t>(мр)</t>
+    </r>
   </si>
   <si>
     <r>
@@ -71,7 +101,7 @@
         <family val="2"/>
         <scheme val="minor"/>
       </rPr>
-      <t xml:space="preserve"> (.м.р)</t>
+      <t xml:space="preserve"> (жр)</t>
     </r>
   </si>
   <si>
@@ -86,56 +116,26 @@
         <family val="2"/>
         <scheme val="minor"/>
       </rPr>
-      <t xml:space="preserve"> (.ж.р)</t>
+      <t xml:space="preserve"> (мр)</t>
     </r>
   </si>
   <si>
-    <t>Они (ж.р.)</t>
-  </si>
-  <si>
-    <t>Они (м.р.)</t>
-  </si>
-  <si>
-    <t>Она</t>
-  </si>
-  <si>
-    <t>Ты (м.р.)</t>
-  </si>
-  <si>
-    <t>Мы</t>
-  </si>
-  <si>
-    <t>Я</t>
-  </si>
-  <si>
-    <t>Вы (ж.р.)</t>
-  </si>
-  <si>
-    <t>Вы обе</t>
-  </si>
-  <si>
-    <t>Вы оба</t>
-  </si>
-  <si>
-    <t>Вы (м.р.)</t>
-  </si>
-  <si>
-    <t>Ты (ж.р.)</t>
-  </si>
-  <si>
-    <r>
-      <t xml:space="preserve">أَنْتُمَا </t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="8"/>
-        <color theme="1"/>
-        <rFont val="Calibri"/>
-        <family val="2"/>
-        <scheme val="minor"/>
-      </rPr>
-      <t>(.м.р)</t>
-    </r>
+    <t>Они (мр)</t>
+  </si>
+  <si>
+    <t>Они (жр)</t>
+  </si>
+  <si>
+    <t>Ты (мр)</t>
+  </si>
+  <si>
+    <t>Вы (мр)</t>
+  </si>
+  <si>
+    <t>Ты (жр)</t>
+  </si>
+  <si>
+    <t>Вы (жр)</t>
   </si>
 </sst>
 </file>
@@ -498,7 +498,7 @@
     </row>
     <row r="2" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A2" t="s">
-        <v>14</v>
+        <v>21</v>
       </c>
       <c r="B2" t="s">
         <v>3</v>
@@ -509,7 +509,7 @@
         <v>2</v>
       </c>
       <c r="B3" t="s">
-        <v>17</v>
+        <v>22</v>
       </c>
     </row>
     <row r="4" spans="1:2" x14ac:dyDescent="0.3">
@@ -517,12 +517,12 @@
         <v>5</v>
       </c>
       <c r="B4" t="s">
-        <v>18</v>
+        <v>13</v>
       </c>
     </row>
     <row r="5" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A5" t="s">
-        <v>15</v>
+        <v>20</v>
       </c>
       <c r="B5" t="s">
         <v>4</v>
@@ -533,7 +533,7 @@
         <v>6</v>
       </c>
       <c r="B6" t="s">
-        <v>16</v>
+        <v>23</v>
       </c>
     </row>
     <row r="7" spans="1:2" x14ac:dyDescent="0.3">
@@ -541,20 +541,20 @@
         <v>7</v>
       </c>
       <c r="B7" t="s">
-        <v>19</v>
+        <v>24</v>
       </c>
     </row>
     <row r="8" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A8" t="s">
-        <v>27</v>
+        <v>19</v>
       </c>
       <c r="B8" t="s">
-        <v>24</v>
+        <v>17</v>
       </c>
     </row>
     <row r="9" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A9" t="s">
-        <v>11</v>
+        <v>10</v>
       </c>
       <c r="B9" t="s">
         <v>25</v>
@@ -570,34 +570,34 @@
     </row>
     <row r="11" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A11" t="s">
-        <v>9</v>
+        <v>18</v>
       </c>
       <c r="B11" t="s">
-        <v>23</v>
+        <v>16</v>
       </c>
     </row>
     <row r="12" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A12" t="s">
-        <v>10</v>
+        <v>9</v>
       </c>
       <c r="B12" t="s">
-        <v>22</v>
+        <v>27</v>
       </c>
     </row>
     <row r="13" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A13" t="s">
-        <v>12</v>
+        <v>11</v>
       </c>
       <c r="B13" t="s">
-        <v>21</v>
+        <v>15</v>
       </c>
     </row>
     <row r="14" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A14" t="s">
-        <v>13</v>
+        <v>12</v>
       </c>
       <c r="B14" t="s">
-        <v>20</v>
+        <v>14</v>
       </c>
     </row>
   </sheetData>

</xml_diff>